<commit_message>
People Requests template: fill sample values so every column imports as text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWpepS9wV9DZhmZr7JVMkV
</commit_message>
<xml_diff>
--- a/altas-bajas/PeopleRequests.xlsx
+++ b/altas-bajas/PeopleRequests.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -52,10 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,7 +619,7 @@
           <t>sperson@sussek.com</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>46328</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -682,10 +682,26 @@
           <t>Quality shared folder</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Job title: Inspector | Department: Quality</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>newmanager@sussek.com</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>newmanager@sussek.com</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Sample Person is no longer with Sussek. Please contact New Manager at newmanager@sussek.com.</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>Delete this sample row after the list is created.</t>

</xml_diff>